<commit_message>
chore(tracker): auto-refresh reconcile + phase-manifest artifacts (#3291)
Co-authored-by: github-actions[bot] <41898282+github-actions[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/trackers/exports/IH35-TMS-BLOCK-RECONCILIATION-2026-07-23.xlsx
+++ b/docs/trackers/exports/IH35-TMS-BLOCK-RECONCILIATION-2026-07-23.xlsx
@@ -14,7 +14,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7166" uniqueCount="1790">
   <si>
-    <t>IH35-TMS — EVERY BLOCK, BUILT vs PENDING — 2026-07-23 (verified vs origin/main + 2991 merged PRs)</t>
+    <t>IH35-TMS — EVERY BLOCK, BUILT vs PENDING — 2026-07-23 (verified vs origin/main + 2994 merged PRs)</t>
   </si>
   <si>
     <t>DONE = verified on main (branch merged or files present) · NEEDS-VERIFY = weak signal, not trusted until GUARD confirms · PENDING = needs build · PENDING (GATED) = financial/locked, needs Jorge's gate first</t>
@@ -29799,7 +29799,7 @@
         <v>1788</v>
       </c>
       <c r="B10">
-        <v>2991</v>
+        <v>2994</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -29807,7 +29807,7 @@
         <v>1789</v>
       </c>
       <c r="B11">
-        <v>10812</v>
+        <v>10819</v>
       </c>
     </row>
   </sheetData>

</xml_diff>